<commit_message>
feat: SPIN导出功能 + Transportation解析 + 多项修复
- SPIN导出: 使用VQ-template-spin.xlsx模板，填充角色sheet数据
  - In-Housed Molding (中英文名)
  - Purchased Part (Fabric/Metal/Electronic/Others，多款式显示款式列)
  - Packaging (Retail box + Master carton)
  - Labor Misc (固定rate from labor_hkd)
  - Transportation (SpinTransportRow数据)
  - Markup/Scrap/Misc Cost/Testing Fee
  - Summary sheet (公式引用修正，纸箱尺寸)
  - Electronic超出10行时用duplicateRow扩展
- Transportation解析: 从主sheet提取盐田/HK FCL和LCL数据
- 解析修复: PP胶粒单价、测试费、纸箱尺寸、item_desc提取
- UI: spin-transport tab、智能分组(getSewingGroups)、Markup显示测试费和纸箱尺寸
- 导入: force_format传给parseWorkbook、client参数、labor_hkd解析
- TOMY: 动态labor/hardware/packaging行号检测

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/templates/VQ-template-spin.xlsx
+++ b/server/templates/VQ-template-spin.xlsx
@@ -5244,288 +5244,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>546735</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>27940</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>132080</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>53975</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="图片 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8684260" y="447040"/>
-          <a:ext cx="1574165" cy="1186180"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>394335</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>5715</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>760095</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>4445</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="图片 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8531860" y="424815"/>
-          <a:ext cx="1546225" cy="1158875"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1082040</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>186690</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>579755</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>8890</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="图片 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9219565" y="415290"/>
-          <a:ext cx="1486535" cy="1172845"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>154940</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>150495</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>737870</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>118110</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="图片 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9472930" y="379095"/>
-          <a:ext cx="1391285" cy="1143000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>131445</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>86995</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>762635</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>83820</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="图片 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9449435" y="315595"/>
-          <a:ext cx="1439545" cy="1172210"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>199390</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>125730</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>796290</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>109855</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="图片 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9517380" y="354330"/>
-          <a:ext cx="1405255" cy="1159510"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
   <a:themeElements>
@@ -15559,7 +15277,6 @@
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="50" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -23849,7 +23566,6 @@
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="50" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -32130,7 +31846,6 @@
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="50" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -40420,7 +40135,6 @@
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="50" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -48701,7 +48415,6 @@
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="50" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -56982,7 +56695,6 @@
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="50" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>